<commit_message>
Reconcile checking to Chase through 9/30 ($2,016.62); $1,828 PayPal as October income
Added Costco gas, ATM, Zelle and GovAuctions; Mr Terrible posted at $7;
UPS holds and Google $19.99 never posted (uncounted). Rebuilt the
September expenses workbook with a reusable report script.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PkDrCxYQg69AVAk2ernwu3
</commit_message>
<xml_diff>
--- a/reports/September_2026_Expenses.xlsx
+++ b/reports/September_2026_Expenses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Line Items" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Line Items'!$A$1:$F$188</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Line Items'!$A$1:$F$189</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="280">
-  <si>
-    <t xml:space="preserve">Perez Household - September 2026 Expenses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cash (checking) and card spending by category. Pulled from the Perez Household Ledger on 10/1/2026.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="283">
+  <si>
+    <t xml:space="preserve">Perez Household - 2026-09 Expenses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash (checking) and card spending by category, from the Perez Household Ledger.</t>
   </si>
   <si>
     <t xml:space="preserve">Group</t>
@@ -125,15 +125,15 @@
     <t xml:space="preserve">Medical</t>
   </si>
   <si>
+    <t xml:space="preserve">Gas</t>
+  </si>
+  <si>
     <t xml:space="preserve">Remittance - Aron</t>
   </si>
   <si>
     <t xml:space="preserve">Food - To go</t>
   </si>
   <si>
-    <t xml:space="preserve">Gas</t>
-  </si>
-  <si>
     <t xml:space="preserve">Groceries - Seafood City</t>
   </si>
   <si>
@@ -149,12 +149,12 @@
     <t xml:space="preserve">Compass</t>
   </si>
   <si>
+    <t xml:space="preserve">Food - Misc</t>
+  </si>
+  <si>
     <t xml:space="preserve">For Car</t>
   </si>
   <si>
-    <t xml:space="preserve">Food - Misc</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total Expenses</t>
   </si>
   <si>
@@ -200,7 +200,61 @@
     <t xml:space="preserve">Check: equals Line Items total</t>
   </si>
   <si>
-    <t xml:space="preserve">Not counted yet (checked off but not posted in Chase as of 9/29) - not included above</t>
+    <t xml:space="preserve">Not counted yet (checked off or held, but not posted in Chase) - not included above</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afterpay - checked off as paid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC - Credit 1 (...4838) - checked off as paid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SW Gas - checked off as paid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Affirm - Wayfair (2nd plan) - installment 1/3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPS shipping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POS DEBIT GOOGLE *G1AI101M G.CO/HELPPAY CA (...5438)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPS ship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total not counted yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Cash = paid from Chase checking (...0861). Card = purchases, fees and interest on credit card statements, by transaction date.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Credit card payments from checking are left out, since the card purchases themselves are counted (no double counting).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Income and transfers (PayPal, savings) are not expenses and are excluded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Debt includes Affirm, Klarna, Chase Pay in 4, auto loans and card fees/interest. Refunds and credits show as negatives.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Card statements only cover purchases through each card's closing date; later purchases appear on the next statements.</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
@@ -209,54 +263,12 @@
     <t xml:space="preserve">Description</t>
   </si>
   <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
     <t xml:space="preserve">Amount</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Afterpay - checked off as paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC - Credit 1 (...4838) - checked off as paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SW Gas - checked off as paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Affirm - Wayfair (2nd plan) - installment 1/3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total not counted yet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Cash = paid from Chase checking (...0861). Card = purchases, fees and interest on credit card statements, by transaction date.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Credit card payments from checking are left out, since the card purchases themselves are counted (no double counting).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Income and transfers (PayPal, savings) are not expenses and are excluded.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Debt includes Affirm, Klarna, Chase Pay in 4, auto loans and card fees/interest. Refunds and credits show as negatives.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Card statements only cover purchases through each card's September closing date; later September card purchases appear on October statements.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-09-01</t>
   </si>
   <si>
@@ -800,15 +812,9 @@
     <t xml:space="preserve">Kitchen USA - foodie las vegas</t>
   </si>
   <si>
-    <t xml:space="preserve">POS DEBIT GOOGLE *G1AI101M G.CO/HELPPAY CA (...5438)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pegs Glorified</t>
   </si>
   <si>
-    <t xml:space="preserve">UPS shipping</t>
-  </si>
-  <si>
     <t xml:space="preserve">Walmart</t>
   </si>
   <si>
@@ -827,15 +833,9 @@
     <t xml:space="preserve">kitchen light</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-29</t>
-  </si>
-  <si>
     <t xml:space="preserve">POS DEBIT MR TERRIBLE SELF-SERV HENDERSON NV</t>
   </si>
   <si>
-    <t xml:space="preserve">UPS ship</t>
-  </si>
-  <si>
     <t xml:space="preserve">auntioe annes</t>
   </si>
   <si>
@@ -848,9 +848,18 @@
     <t xml:space="preserve">zelle to buy pickleball</t>
   </si>
   <si>
+    <t xml:space="preserve">ATM WITHDRAWAL 005706 09/30</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dam Roast</t>
   </si>
   <si>
+    <t xml:space="preserve">PAYPAL PURCHASE GOVAUCTIONS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zelle payment to Mary Gerbino JPM99cy9d01s</t>
+  </si>
+  <si>
     <t xml:space="preserve">amazon - filter for dyson</t>
   </si>
   <si>
@@ -863,7 +872,7 @@
     <t xml:space="preserve">zelle - mattress</t>
   </si>
   <si>
-    <t xml:space="preserve">Amounts are money spent (positive). Refunds and credits are negative. Card rows are purchases, fees and interest from card statements; checking payments to those cards are left out so nothing is counted twice.</t>
+    <t xml:space="preserve">Amounts are money spent (positive); refunds and credits are negative. Card rows are purchases, fees and interest from card statements; checking payments to those cards are left out so nothing is counted twice.</t>
   </si>
 </sst>
 </file>
@@ -1366,7 +1375,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -1409,11 +1418,11 @@
         <v>8</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A5,'Line Items'!$E$2:$E$188,$B5,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A5,'Line Items'!$E$2:$E$189,$B5,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>278.91</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A5,'Line Items'!$E$2:$E$188,$B5,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A5,'Line Items'!$E$2:$E$189,$B5,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>310.89</v>
       </c>
       <c r="E5" s="5" t="n">
@@ -1429,11 +1438,11 @@
         <v>9</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A6,'Line Items'!$E$2:$E$188,$B6,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A6,'Line Items'!$E$2:$E$189,$B6,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>401.75</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A6,'Line Items'!$E$2:$E$188,$B6,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A6,'Line Items'!$E$2:$E$189,$B6,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E6" s="5" t="n">
@@ -1449,11 +1458,11 @@
         <v>10</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A7,'Line Items'!$E$2:$E$188,$B7,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A7,'Line Items'!$E$2:$E$189,$B7,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>289.55</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A7,'Line Items'!$E$2:$E$188,$B7,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A7,'Line Items'!$E$2:$E$189,$B7,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
@@ -1469,11 +1478,11 @@
         <v>11</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A8,'Line Items'!$E$2:$E$188,$B8,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A8,'Line Items'!$E$2:$E$189,$B8,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>205.62</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A8,'Line Items'!$E$2:$E$188,$B8,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A8,'Line Items'!$E$2:$E$189,$B8,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
@@ -1489,11 +1498,11 @@
         <v>12</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A9,'Line Items'!$E$2:$E$188,$B9,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A9,'Line Items'!$E$2:$E$189,$B9,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>200</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A9,'Line Items'!$E$2:$E$188,$B9,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A9,'Line Items'!$E$2:$E$189,$B9,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
@@ -1509,11 +1518,11 @@
         <v>13</v>
       </c>
       <c r="C10" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A10,'Line Items'!$E$2:$E$188,$B10,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A10,'Line Items'!$E$2:$E$189,$B10,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>130</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A10,'Line Items'!$E$2:$E$188,$B10,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A10,'Line Items'!$E$2:$E$189,$B10,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E10" s="5" t="n">
@@ -1529,11 +1538,11 @@
         <v>14</v>
       </c>
       <c r="C11" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A11,'Line Items'!$E$2:$E$188,$B11,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A11,'Line Items'!$E$2:$E$189,$B11,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>93.31</v>
       </c>
       <c r="D11" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A11,'Line Items'!$E$2:$E$188,$B11,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A11,'Line Items'!$E$2:$E$189,$B11,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E11" s="5" t="n">
@@ -1549,11 +1558,11 @@
         <v>15</v>
       </c>
       <c r="C12" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A12,'Line Items'!$E$2:$E$188,$B12,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A12,'Line Items'!$E$2:$E$189,$B12,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>59.67</v>
       </c>
       <c r="D12" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A12,'Line Items'!$E$2:$E$188,$B12,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A12,'Line Items'!$E$2:$E$189,$B12,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E12" s="5" t="n">
@@ -1569,11 +1578,11 @@
         <v>16</v>
       </c>
       <c r="C13" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A13,'Line Items'!$E$2:$E$188,$B13,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A13,'Line Items'!$E$2:$E$189,$B13,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>49.72</v>
       </c>
       <c r="D13" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A13,'Line Items'!$E$2:$E$188,$B13,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A13,'Line Items'!$E$2:$E$189,$B13,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
@@ -1589,11 +1598,11 @@
         <v>17</v>
       </c>
       <c r="C14" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A14,'Line Items'!$E$2:$E$188,$B14,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A14,'Line Items'!$E$2:$E$189,$B14,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>48.96</v>
       </c>
       <c r="D14" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A14,'Line Items'!$E$2:$E$188,$B14,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A14,'Line Items'!$E$2:$E$189,$B14,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E14" s="5" t="n">
@@ -1609,11 +1618,11 @@
         <v>18</v>
       </c>
       <c r="C15" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A15,'Line Items'!$E$2:$E$188,$B15,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A15,'Line Items'!$E$2:$E$189,$B15,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>29.98</v>
       </c>
       <c r="D15" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A15,'Line Items'!$E$2:$E$188,$B15,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A15,'Line Items'!$E$2:$E$189,$B15,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E15" s="5" t="n">
@@ -1629,11 +1638,11 @@
         <v>19</v>
       </c>
       <c r="C16" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A16,'Line Items'!$E$2:$E$188,$B16,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A16,'Line Items'!$E$2:$E$189,$B16,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>14.99</v>
       </c>
       <c r="D16" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A16,'Line Items'!$E$2:$E$188,$B16,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A16,'Line Items'!$E$2:$E$189,$B16,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E16" s="5" t="n">
@@ -1649,11 +1658,11 @@
         <v>20</v>
       </c>
       <c r="C17" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A17,'Line Items'!$E$2:$E$188,$B17,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A17,'Line Items'!$E$2:$E$189,$B17,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>14.39</v>
       </c>
       <c r="D17" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A17,'Line Items'!$E$2:$E$188,$B17,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A17,'Line Items'!$E$2:$E$189,$B17,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
@@ -1669,11 +1678,11 @@
         <v>21</v>
       </c>
       <c r="C18" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A18,'Line Items'!$E$2:$E$188,$B18,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A18,'Line Items'!$E$2:$E$189,$B18,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>13.99</v>
       </c>
       <c r="D18" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A18,'Line Items'!$E$2:$E$188,$B18,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A18,'Line Items'!$E$2:$E$189,$B18,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E18" s="5" t="n">
@@ -1689,11 +1698,11 @@
         <v>22</v>
       </c>
       <c r="C19" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A19,'Line Items'!$E$2:$E$188,$B19,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A19,'Line Items'!$E$2:$E$189,$B19,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>13.49</v>
       </c>
       <c r="D19" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A19,'Line Items'!$E$2:$E$188,$B19,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A19,'Line Items'!$E$2:$E$189,$B19,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E19" s="5" t="n">
@@ -1732,16 +1741,16 @@
         <v>25</v>
       </c>
       <c r="C22" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A22,'Line Items'!$E$2:$E$188,$B22,'Line Items'!$C$2:$C$188,"Checking")</f>
-        <v>2850.88</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A22,'Line Items'!$E$2:$E$189,$B22,'Line Items'!$C$2:$C$189,"Checking")</f>
+        <v>2758.44</v>
       </c>
       <c r="D22" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A22,'Line Items'!$E$2:$E$188,$B22,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A22,'Line Items'!$E$2:$E$189,$B22,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>30</v>
       </c>
       <c r="E22" s="5" t="n">
         <f aca="false">C22+D22</f>
-        <v>2880.88</v>
+        <v>2788.44</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1752,11 +1761,11 @@
         <v>26</v>
       </c>
       <c r="C23" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A23,'Line Items'!$E$2:$E$188,$B23,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A23,'Line Items'!$E$2:$E$189,$B23,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>1280.67</v>
       </c>
       <c r="D23" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A23,'Line Items'!$E$2:$E$188,$B23,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A23,'Line Items'!$E$2:$E$189,$B23,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E23" s="5" t="n">
@@ -1772,11 +1781,11 @@
         <v>27</v>
       </c>
       <c r="C24" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A24,'Line Items'!$E$2:$E$188,$B24,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A24,'Line Items'!$E$2:$E$189,$B24,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>762.18</v>
       </c>
       <c r="D24" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A24,'Line Items'!$E$2:$E$188,$B24,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A24,'Line Items'!$E$2:$E$189,$B24,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E24" s="5" t="n">
@@ -1792,11 +1801,11 @@
         <v>28</v>
       </c>
       <c r="C25" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A25,'Line Items'!$E$2:$E$188,$B25,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A25,'Line Items'!$E$2:$E$189,$B25,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>741.55</v>
       </c>
       <c r="D25" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A25,'Line Items'!$E$2:$E$188,$B25,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A25,'Line Items'!$E$2:$E$189,$B25,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E25" s="5" t="n">
@@ -1812,11 +1821,11 @@
         <v>29</v>
       </c>
       <c r="C26" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A26,'Line Items'!$E$2:$E$188,$B26,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A26,'Line Items'!$E$2:$E$189,$B26,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>469.52</v>
       </c>
       <c r="D26" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A26,'Line Items'!$E$2:$E$188,$B26,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A26,'Line Items'!$E$2:$E$189,$B26,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E26" s="5" t="n">
@@ -1832,11 +1841,11 @@
         <v>30</v>
       </c>
       <c r="C27" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A27,'Line Items'!$E$2:$E$188,$B27,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A27,'Line Items'!$E$2:$E$189,$B27,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>331.53</v>
       </c>
       <c r="D27" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A27,'Line Items'!$E$2:$E$188,$B27,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A27,'Line Items'!$E$2:$E$189,$B27,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>53.38</v>
       </c>
       <c r="E27" s="5" t="n">
@@ -1852,11 +1861,11 @@
         <v>31</v>
       </c>
       <c r="C28" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A28,'Line Items'!$E$2:$E$188,$B28,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A28,'Line Items'!$E$2:$E$189,$B28,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D28" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A28,'Line Items'!$E$2:$E$188,$B28,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A28,'Line Items'!$E$2:$E$189,$B28,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>331</v>
       </c>
       <c r="E28" s="5" t="n">
@@ -1872,11 +1881,11 @@
         <v>32</v>
       </c>
       <c r="C29" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A29,'Line Items'!$E$2:$E$188,$B29,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A29,'Line Items'!$E$2:$E$189,$B29,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>21.66</v>
       </c>
       <c r="D29" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A29,'Line Items'!$E$2:$E$188,$B29,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A29,'Line Items'!$E$2:$E$189,$B29,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>304.42</v>
       </c>
       <c r="E29" s="5" t="n">
@@ -1892,16 +1901,16 @@
         <v>33</v>
       </c>
       <c r="C30" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A30,'Line Items'!$E$2:$E$188,$B30,'Line Items'!$C$2:$C$188,"Checking")</f>
-        <v>242.45</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A30,'Line Items'!$E$2:$E$189,$B30,'Line Items'!$C$2:$C$189,"Checking")</f>
+        <v>211.4</v>
       </c>
       <c r="D30" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A30,'Line Items'!$E$2:$E$188,$B30,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
-        <v>0</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A30,'Line Items'!$E$2:$E$189,$B30,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
+        <v>67.49</v>
       </c>
       <c r="E30" s="5" t="n">
         <f aca="false">C30+D30</f>
-        <v>242.45</v>
+        <v>278.89</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1912,16 +1921,16 @@
         <v>34</v>
       </c>
       <c r="C31" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A31,'Line Items'!$E$2:$E$188,$B31,'Line Items'!$C$2:$C$188,"Checking")</f>
-        <v>232.71</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A31,'Line Items'!$E$2:$E$189,$B31,'Line Items'!$C$2:$C$189,"Checking")</f>
+        <v>242.45</v>
       </c>
       <c r="D31" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A31,'Line Items'!$E$2:$E$188,$B31,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A31,'Line Items'!$E$2:$E$189,$B31,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E31" s="5" t="n">
         <f aca="false">C31+D31</f>
-        <v>232.71</v>
+        <v>242.45</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1932,16 +1941,16 @@
         <v>35</v>
       </c>
       <c r="C32" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A32,'Line Items'!$E$2:$E$188,$B32,'Line Items'!$C$2:$C$188,"Checking")</f>
-        <v>133.08</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A32,'Line Items'!$E$2:$E$189,$B32,'Line Items'!$C$2:$C$189,"Checking")</f>
+        <v>232.71</v>
       </c>
       <c r="D32" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A32,'Line Items'!$E$2:$E$188,$B32,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
-        <v>67.49</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A32,'Line Items'!$E$2:$E$189,$B32,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
+        <v>0</v>
       </c>
       <c r="E32" s="5" t="n">
         <f aca="false">C32+D32</f>
-        <v>200.57</v>
+        <v>232.71</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1952,11 +1961,11 @@
         <v>36</v>
       </c>
       <c r="C33" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A33,'Line Items'!$E$2:$E$188,$B33,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A33,'Line Items'!$E$2:$E$189,$B33,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>175.94</v>
       </c>
       <c r="D33" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A33,'Line Items'!$E$2:$E$188,$B33,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A33,'Line Items'!$E$2:$E$189,$B33,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E33" s="5" t="n">
@@ -1972,11 +1981,11 @@
         <v>37</v>
       </c>
       <c r="C34" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A34,'Line Items'!$E$2:$E$188,$B34,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A34,'Line Items'!$E$2:$E$189,$B34,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>93.04</v>
       </c>
       <c r="D34" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A34,'Line Items'!$E$2:$E$188,$B34,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A34,'Line Items'!$E$2:$E$189,$B34,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E34" s="5" t="n">
@@ -1992,11 +2001,11 @@
         <v>38</v>
       </c>
       <c r="C35" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A35,'Line Items'!$E$2:$E$188,$B35,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A35,'Line Items'!$E$2:$E$189,$B35,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>47.93</v>
       </c>
       <c r="D35" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A35,'Line Items'!$E$2:$E$188,$B35,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A35,'Line Items'!$E$2:$E$189,$B35,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E35" s="5" t="n">
@@ -2012,11 +2021,11 @@
         <v>39</v>
       </c>
       <c r="C36" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A36,'Line Items'!$E$2:$E$188,$B36,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A36,'Line Items'!$E$2:$E$189,$B36,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D36" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A36,'Line Items'!$E$2:$E$188,$B36,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A36,'Line Items'!$E$2:$E$189,$B36,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>40</v>
       </c>
       <c r="E36" s="5" t="n">
@@ -2032,11 +2041,11 @@
         <v>40</v>
       </c>
       <c r="C37" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A37,'Line Items'!$E$2:$E$188,$B37,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A37,'Line Items'!$E$2:$E$189,$B37,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>40</v>
       </c>
       <c r="D37" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A37,'Line Items'!$E$2:$E$188,$B37,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A37,'Line Items'!$E$2:$E$189,$B37,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E37" s="5" t="n">
@@ -2052,16 +2061,16 @@
         <v>41</v>
       </c>
       <c r="C38" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A38,'Line Items'!$E$2:$E$188,$B38,'Line Items'!$C$2:$C$188,"Checking")</f>
-        <v>15</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A38,'Line Items'!$E$2:$E$189,$B38,'Line Items'!$C$2:$C$189,"Checking")</f>
+        <v>7.8</v>
       </c>
       <c r="D38" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A38,'Line Items'!$E$2:$E$188,$B38,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A38,'Line Items'!$E$2:$E$189,$B38,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E38" s="5" t="n">
         <f aca="false">C38+D38</f>
-        <v>15</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2072,16 +2081,16 @@
         <v>42</v>
       </c>
       <c r="C39" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A39,'Line Items'!$E$2:$E$188,$B39,'Line Items'!$C$2:$C$188,"Checking")</f>
-        <v>7.8</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A39,'Line Items'!$E$2:$E$189,$B39,'Line Items'!$C$2:$C$189,"Checking")</f>
+        <v>7</v>
       </c>
       <c r="D39" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A39,'Line Items'!$E$2:$E$188,$B39,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A39,'Line Items'!$E$2:$E$189,$B39,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E39" s="5" t="n">
         <f aca="false">C39+D39</f>
-        <v>7.8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2091,7 +2100,7 @@
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="n">
         <f aca="false">SUM(C22:C39)</f>
-        <v>7445.94</v>
+        <v>7423.82</v>
       </c>
       <c r="D40" s="7" t="n">
         <f aca="false">SUM(D22:D39)</f>
@@ -2099,7 +2108,7 @@
       </c>
       <c r="E40" s="7" t="n">
         <f aca="false">SUM(E22:E39)</f>
-        <v>8272.23</v>
+        <v>8250.11</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2115,11 +2124,11 @@
         <v>45</v>
       </c>
       <c r="C42" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A42,'Line Items'!$E$2:$E$188,$B42,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A42,'Line Items'!$E$2:$E$189,$B42,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>1081.38</v>
       </c>
       <c r="D42" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A42,'Line Items'!$E$2:$E$188,$B42,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A42,'Line Items'!$E$2:$E$189,$B42,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E42" s="5" t="n">
@@ -2135,11 +2144,11 @@
         <v>46</v>
       </c>
       <c r="C43" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A43,'Line Items'!$E$2:$E$188,$B43,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A43,'Line Items'!$E$2:$E$189,$B43,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>709.9</v>
       </c>
       <c r="D43" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A43,'Line Items'!$E$2:$E$188,$B43,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A43,'Line Items'!$E$2:$E$189,$B43,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E43" s="5" t="n">
@@ -2155,11 +2164,11 @@
         <v>47</v>
       </c>
       <c r="C44" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A44,'Line Items'!$E$2:$E$188,$B44,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A44,'Line Items'!$E$2:$E$189,$B44,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>706.36</v>
       </c>
       <c r="D44" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A44,'Line Items'!$E$2:$E$188,$B44,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A44,'Line Items'!$E$2:$E$189,$B44,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E44" s="5" t="n">
@@ -2175,11 +2184,11 @@
         <v>48</v>
       </c>
       <c r="C45" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A45,'Line Items'!$E$2:$E$188,$B45,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A45,'Line Items'!$E$2:$E$189,$B45,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>500</v>
       </c>
       <c r="D45" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A45,'Line Items'!$E$2:$E$188,$B45,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A45,'Line Items'!$E$2:$E$189,$B45,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E45" s="5" t="n">
@@ -2195,11 +2204,11 @@
         <v>49</v>
       </c>
       <c r="C46" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A46,'Line Items'!$E$2:$E$188,$B46,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A46,'Line Items'!$E$2:$E$189,$B46,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>214.19</v>
       </c>
       <c r="D46" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A46,'Line Items'!$E$2:$E$188,$B46,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A46,'Line Items'!$E$2:$E$189,$B46,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E46" s="5" t="n">
@@ -2215,11 +2224,11 @@
         <v>50</v>
       </c>
       <c r="C47" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A47,'Line Items'!$E$2:$E$188,$B47,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A47,'Line Items'!$E$2:$E$189,$B47,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>150.4</v>
       </c>
       <c r="D47" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A47,'Line Items'!$E$2:$E$188,$B47,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A47,'Line Items'!$E$2:$E$189,$B47,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E47" s="5" t="n">
@@ -2235,11 +2244,11 @@
         <v>51</v>
       </c>
       <c r="C48" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A48,'Line Items'!$E$2:$E$188,$B48,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A48,'Line Items'!$E$2:$E$189,$B48,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D48" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A48,'Line Items'!$E$2:$E$188,$B48,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A48,'Line Items'!$E$2:$E$189,$B48,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>46.5</v>
       </c>
       <c r="E48" s="5" t="n">
@@ -2255,11 +2264,11 @@
         <v>52</v>
       </c>
       <c r="C49" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A49,'Line Items'!$E$2:$E$188,$B49,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A49,'Line Items'!$E$2:$E$189,$B49,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D49" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A49,'Line Items'!$E$2:$E$188,$B49,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A49,'Line Items'!$E$2:$E$189,$B49,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>27</v>
       </c>
       <c r="E49" s="5" t="n">
@@ -2275,11 +2284,11 @@
         <v>53</v>
       </c>
       <c r="C50" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A50,'Line Items'!$E$2:$E$188,$B50,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A50,'Line Items'!$E$2:$E$189,$B50,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D50" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A50,'Line Items'!$E$2:$E$188,$B50,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A50,'Line Items'!$E$2:$E$189,$B50,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>15.9</v>
       </c>
       <c r="E50" s="5" t="n">
@@ -2295,11 +2304,11 @@
         <v>54</v>
       </c>
       <c r="C51" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A51,'Line Items'!$E$2:$E$188,$B51,'Line Items'!$C$2:$C$188,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A51,'Line Items'!$E$2:$E$189,$B51,'Line Items'!$C$2:$C$189,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D51" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$188,'Line Items'!$D$2:$D$188,$A51,'Line Items'!$E$2:$E$188,$B51,'Line Items'!$C$2:$C$188,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$189,'Line Items'!$D$2:$D$189,$A51,'Line Items'!$E$2:$E$189,$B51,'Line Items'!$C$2:$C$189,"&lt;&gt;Checking")</f>
         <v>5.68</v>
       </c>
       <c r="E51" s="5" t="n">
@@ -2337,7 +2346,7 @@
       <c r="B54" s="9"/>
       <c r="C54" s="10" t="n">
         <f aca="false">C20+C40+C52</f>
-        <v>12652.5</v>
+        <v>12630.38</v>
       </c>
       <c r="D54" s="10" t="n">
         <f aca="false">D20+D40+D52</f>
@@ -2345,7 +2354,7 @@
       </c>
       <c r="E54" s="10" t="n">
         <f aca="false">E20+E40+E52</f>
-        <v>13884.76</v>
+        <v>13862.64</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2353,7 +2362,7 @@
         <v>57</v>
       </c>
       <c r="E55" s="2" t="str">
-        <f aca="false">IF(ROUND(E54-'Line Items'!F189,2)=0,"OK","MISMATCH")</f>
+        <f aca="false">IF(ROUND(E54-'Line Items'!F190,2)=0,"OK","MISMATCH")</f>
         <v>OK</v>
       </c>
     </row>
@@ -2363,36 +2372,36 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E58" s="11" t="s">
-        <v>61</v>
+      <c r="E58" s="5" t="n">
+        <v>10.74</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>63</v>
-      </c>
       <c r="E59" s="5" t="n">
-        <v>10.74</v>
+        <v>24.94</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E60" s="5" t="n">
-        <v>24.94</v>
+        <v>13.06</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2400,60 +2409,82 @@
         <v>64</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>13.06</v>
+        <v>39.33</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E62" s="5" t="n">
+        <v>130.88</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B63" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="E63" s="5" t="n">
+        <v>19.99</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E62" s="5" t="n">
-        <v>39.33</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="11" t="s">
+      <c r="B64" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E63" s="12" t="n">
-        <f aca="false">SUM(E59:E62)</f>
-        <v>88.07</v>
+      <c r="E64" s="5" t="n">
+        <v>11.58</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="13" t="s">
+      <c r="B65" s="11" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="14" t="s">
+      <c r="E65" s="12" t="n">
+        <f aca="false">SUM(E58:E64)</f>
+        <v>250.52</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="13" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="14" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="14" t="s">
         <v>75</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="14" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2472,7 +2503,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F191"/>
+  <dimension ref="A1:F192"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -2485,13 +2516,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -2500,24 +2531,24 @@
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>39.41</v>
@@ -2525,13 +2556,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>24</v>
@@ -2545,19 +2576,19 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>80.45</v>
@@ -2565,19 +2596,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>80.64</v>
@@ -2585,13 +2616,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>24</v>
@@ -2605,13 +2636,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>24</v>
@@ -2625,13 +2656,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>24</v>
@@ -2645,13 +2676,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>24</v>
@@ -2665,13 +2696,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>24</v>
@@ -2685,13 +2716,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>24</v>
@@ -2705,13 +2736,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>24</v>
@@ -2725,13 +2756,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>24</v>
@@ -2745,13 +2776,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>24</v>
@@ -2765,13 +2796,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>24</v>
@@ -2785,13 +2816,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>24</v>
@@ -2805,13 +2836,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>24</v>
@@ -2825,13 +2856,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>24</v>
@@ -2845,13 +2876,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>24</v>
@@ -2865,13 +2896,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>24</v>
@@ -2885,13 +2916,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>24</v>
@@ -2905,13 +2936,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>24</v>
@@ -2925,13 +2956,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>24</v>
@@ -2945,13 +2976,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>24</v>
@@ -2965,13 +2996,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>24</v>
@@ -2985,13 +3016,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>44</v>
@@ -3005,13 +3036,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>24</v>
@@ -3025,13 +3056,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>24</v>
@@ -3045,13 +3076,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>24</v>
@@ -3065,13 +3096,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>24</v>
@@ -3085,13 +3116,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>44</v>
@@ -3105,13 +3136,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>44</v>
@@ -3125,13 +3156,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>44</v>
@@ -3145,19 +3176,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F34" s="5" t="n">
         <v>67.49</v>
@@ -3165,13 +3196,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>24</v>
@@ -3185,13 +3216,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>24</v>
@@ -3205,13 +3236,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>24</v>
@@ -3225,13 +3256,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>24</v>
@@ -3245,13 +3276,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>7</v>
@@ -3265,13 +3296,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>44</v>
@@ -3285,13 +3316,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>24</v>
@@ -3305,13 +3336,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>24</v>
@@ -3325,13 +3356,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>24</v>
@@ -3345,13 +3376,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>24</v>
@@ -3365,13 +3396,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>24</v>
@@ -3385,13 +3416,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>24</v>
@@ -3405,13 +3436,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>24</v>
@@ -3425,13 +3456,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>24</v>
@@ -3445,13 +3476,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>7</v>
@@ -3465,13 +3496,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>24</v>
@@ -3485,13 +3516,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>24</v>
@@ -3505,13 +3536,13 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>44</v>
@@ -3525,13 +3556,13 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>24</v>
@@ -3545,13 +3576,13 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>24</v>
@@ -3565,13 +3596,13 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>24</v>
@@ -3585,13 +3616,13 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>7</v>
@@ -3605,13 +3636,13 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>24</v>
@@ -3625,13 +3656,13 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>24</v>
@@ -3645,13 +3676,13 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>24</v>
@@ -3665,13 +3696,13 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>24</v>
@@ -3685,13 +3716,13 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>24</v>
@@ -3705,13 +3736,13 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>24</v>
@@ -3725,13 +3756,13 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>24</v>
@@ -3745,13 +3776,13 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>7</v>
@@ -3765,13 +3796,13 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>24</v>
@@ -3785,13 +3816,13 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>24</v>
@@ -3805,13 +3836,13 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>24</v>
@@ -3825,13 +3856,13 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>24</v>
@@ -3845,13 +3876,13 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>24</v>
@@ -3865,13 +3896,13 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>44</v>
@@ -3885,13 +3916,13 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>24</v>
@@ -3905,13 +3936,13 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>44</v>
@@ -3925,13 +3956,13 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>24</v>
@@ -3945,13 +3976,13 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>44</v>
@@ -3965,13 +3996,13 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>24</v>
@@ -3985,13 +4016,13 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>24</v>
@@ -4005,13 +4036,13 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>24</v>
@@ -4025,13 +4056,13 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>7</v>
@@ -4045,13 +4076,13 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>24</v>
@@ -4065,19 +4096,19 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F80" s="5" t="n">
         <v>52.63</v>
@@ -4085,13 +4116,13 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>44</v>
@@ -4105,13 +4136,13 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>24</v>
@@ -4125,13 +4156,13 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>44</v>
@@ -4145,13 +4176,13 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>24</v>
@@ -4165,13 +4196,13 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>24</v>
@@ -4185,13 +4216,13 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>24</v>
@@ -4205,13 +4236,13 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>24</v>
@@ -4225,13 +4256,13 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D88" s="4" t="s">
         <v>24</v>
@@ -4245,13 +4276,13 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>24</v>
@@ -4265,13 +4296,13 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>24</v>
@@ -4285,13 +4316,13 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>44</v>
@@ -4305,13 +4336,13 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>24</v>
@@ -4325,13 +4356,13 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>7</v>
@@ -4345,13 +4376,13 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>24</v>
@@ -4365,13 +4396,13 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D95" s="4" t="s">
         <v>24</v>
@@ -4385,13 +4416,13 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>24</v>
@@ -4405,13 +4436,13 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>24</v>
@@ -4425,13 +4456,13 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>24</v>
@@ -4445,13 +4476,13 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>24</v>
@@ -4465,13 +4496,13 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>7</v>
@@ -4485,13 +4516,13 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>7</v>
@@ -4505,13 +4536,13 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D102" s="4" t="s">
         <v>24</v>
@@ -4525,13 +4556,13 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="4" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D103" s="4" t="s">
         <v>24</v>
@@ -4545,13 +4576,13 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D104" s="4" t="s">
         <v>24</v>
@@ -4565,13 +4596,13 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D105" s="4" t="s">
         <v>24</v>
@@ -4585,13 +4616,13 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>24</v>
@@ -4605,13 +4636,13 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>24</v>
@@ -4625,13 +4656,13 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D108" s="4" t="s">
         <v>24</v>
@@ -4645,13 +4676,13 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D109" s="4" t="s">
         <v>7</v>
@@ -4665,13 +4696,13 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D110" s="4" t="s">
         <v>44</v>
@@ -4685,13 +4716,13 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D111" s="4" t="s">
         <v>44</v>
@@ -4705,13 +4736,13 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D112" s="4" t="s">
         <v>44</v>
@@ -4725,13 +4756,13 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D113" s="4" t="s">
         <v>24</v>
@@ -4745,13 +4776,13 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D114" s="4" t="s">
         <v>24</v>
@@ -4765,13 +4796,13 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D115" s="4" t="s">
         <v>24</v>
@@ -4785,19 +4816,19 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D116" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F116" s="5" t="n">
         <v>59.91</v>
@@ -4805,13 +4836,13 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B117" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>24</v>
@@ -4825,13 +4856,13 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D118" s="4" t="s">
         <v>24</v>
@@ -4845,13 +4876,13 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>24</v>
@@ -4865,13 +4896,13 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>44</v>
@@ -4885,13 +4916,13 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="4" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D121" s="4" t="s">
         <v>44</v>
@@ -4905,19 +4936,19 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="4" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D122" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F122" s="5" t="n">
         <v>36.87</v>
@@ -4925,19 +4956,19 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="4" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F123" s="5" t="n">
         <v>51.05</v>
@@ -4945,13 +4976,13 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="4" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D124" s="4" t="s">
         <v>24</v>
@@ -4965,13 +4996,13 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="4" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>24</v>
@@ -4985,13 +5016,13 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>44</v>
@@ -5005,13 +5036,13 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D127" s="4" t="s">
         <v>7</v>
@@ -5025,13 +5056,13 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D128" s="4" t="s">
         <v>7</v>
@@ -5045,13 +5076,13 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D129" s="4" t="s">
         <v>24</v>
@@ -5065,13 +5096,13 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D130" s="4" t="s">
         <v>24</v>
@@ -5085,13 +5116,13 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D131" s="4" t="s">
         <v>24</v>
@@ -5105,13 +5136,13 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D132" s="4" t="s">
         <v>24</v>
@@ -5125,13 +5156,13 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D133" s="4" t="s">
         <v>24</v>
@@ -5145,13 +5176,13 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D134" s="4" t="s">
         <v>24</v>
@@ -5165,13 +5196,13 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D135" s="4" t="s">
         <v>7</v>
@@ -5185,13 +5216,13 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="4" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D136" s="4" t="s">
         <v>24</v>
@@ -5205,13 +5236,13 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="4" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>24</v>
@@ -5225,13 +5256,13 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D138" s="4" t="s">
         <v>24</v>
@@ -5245,13 +5276,13 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D139" s="4" t="s">
         <v>7</v>
@@ -5265,13 +5296,13 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D140" s="4" t="s">
         <v>7</v>
@@ -5285,13 +5316,13 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>24</v>
@@ -5305,13 +5336,13 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D142" s="4" t="s">
         <v>24</v>
@@ -5325,19 +5356,19 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D143" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E143" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F143" s="5" t="n">
         <v>45.47</v>
@@ -5345,13 +5376,13 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D144" s="4" t="s">
         <v>24</v>
@@ -5365,13 +5396,13 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D145" s="4" t="s">
         <v>24</v>
@@ -5385,13 +5416,13 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D146" s="4" t="s">
         <v>24</v>
@@ -5405,13 +5436,13 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="4" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D147" s="4" t="s">
         <v>44</v>
@@ -5425,13 +5456,13 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="4" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D148" s="4" t="s">
         <v>24</v>
@@ -5445,13 +5476,13 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="4" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D149" s="4" t="s">
         <v>24</v>
@@ -5465,13 +5496,13 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D150" s="4" t="s">
         <v>44</v>
@@ -5485,13 +5516,13 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D151" s="4" t="s">
         <v>7</v>
@@ -5505,13 +5536,13 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D152" s="4" t="s">
         <v>7</v>
@@ -5525,13 +5556,13 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D153" s="4" t="s">
         <v>24</v>
@@ -5545,13 +5576,13 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D154" s="4" t="s">
         <v>24</v>
@@ -5565,13 +5596,13 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D155" s="4" t="s">
         <v>24</v>
@@ -5585,13 +5616,13 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D156" s="4" t="s">
         <v>44</v>
@@ -5605,13 +5636,13 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D157" s="4" t="s">
         <v>44</v>
@@ -5625,13 +5656,13 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B158" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D158" s="4" t="s">
         <v>7</v>
@@ -5645,13 +5676,13 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D159" s="4" t="s">
         <v>7</v>
@@ -5665,13 +5696,13 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D160" s="4" t="s">
         <v>24</v>
@@ -5685,13 +5716,13 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D161" s="4" t="s">
         <v>24</v>
@@ -5705,13 +5736,13 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D162" s="4" t="s">
         <v>44</v>
@@ -5725,13 +5756,13 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D163" s="4" t="s">
         <v>24</v>
@@ -5745,13 +5776,13 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D164" s="4" t="s">
         <v>24</v>
@@ -5765,13 +5796,13 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D165" s="4" t="s">
         <v>24</v>
@@ -5785,13 +5816,13 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D166" s="4" t="s">
         <v>24</v>
@@ -5805,13 +5836,13 @@
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D167" s="4" t="s">
         <v>24</v>
@@ -5825,133 +5856,133 @@
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D168" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E168" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F168" s="5" t="n">
-        <v>19.99</v>
+        <v>81.76</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="C169" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D169" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E169" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F169" s="5" t="n">
-        <v>81.76</v>
+        <v>94.83</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C170" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D170" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E170" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F170" s="5" t="n">
-        <v>130.88</v>
+        <v>165.82</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D171" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E171" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F171" s="5" t="n">
-        <v>94.83</v>
+        <v>29.25</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D172" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E172" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F172" s="5" t="n">
-        <v>165.82</v>
+        <v>-180.49</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D173" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E173" s="4" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="F173" s="5" t="n">
-        <v>29.25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D174" s="4" t="s">
         <v>24</v>
@@ -5960,305 +5991,325 @@
         <v>25</v>
       </c>
       <c r="F174" s="5" t="n">
-        <v>-180.49</v>
+        <v>30</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D175" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E175" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F175" s="5" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D176" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E176" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F176" s="5" t="n">
-        <v>30</v>
+        <v>40.86</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="4" t="s">
-        <v>267</v>
+        <v>68</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D177" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E177" s="4" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="F177" s="5" t="n">
-        <v>15</v>
+        <v>55.29</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="4" t="s">
-        <v>267</v>
+        <v>68</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D178" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E178" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F178" s="5" t="n">
-        <v>11.58</v>
+        <v>34.84</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="4" t="s">
-        <v>267</v>
+        <v>68</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D179" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E179" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="F179" s="5" t="n">
-        <v>40.86</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="4" t="s">
-        <v>267</v>
+        <v>68</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D180" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E180" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F180" s="5" t="n">
-        <v>55.29</v>
+        <v>55</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="4" t="s">
-        <v>267</v>
+        <v>64</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D181" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E181" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F181" s="5" t="n">
-        <v>34.84</v>
+        <v>60</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="4" t="s">
-        <v>267</v>
+        <v>64</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>272</v>
+        <v>122</v>
       </c>
       <c r="C182" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D182" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E182" s="4" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F182" s="5" t="n">
-        <v>7.8</v>
+        <v>78.32</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="4" t="s">
-        <v>267</v>
+        <v>64</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D183" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E183" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F183" s="5" t="n">
-        <v>55</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D184" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E184" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>31.8</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D185" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E185" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>30.33</v>
+        <v>10</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D186" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E186" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>9.99</v>
+        <v>30.33</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D187" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E187" s="4" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F187" s="5" t="n">
-        <v>161.81</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D188" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E188" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F188" s="5" t="n">
+        <v>161.81</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B189" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="C189" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D189" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E189" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F188" s="5" t="n">
+      <c r="F189" s="5" t="n">
         <v>125</v>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E189" s="11" t="s">
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E190" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F189" s="12" t="n">
-        <f aca="false">SUM(F2:F188)</f>
-        <v>13884.76</v>
-      </c>
-    </row>
-    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A191" s="2" t="s">
-        <v>279</v>
+      <c r="F190" s="12" t="n">
+        <f aca="false">SUM(F2:F189)</f>
+        <v>13862.64</v>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="2" t="s">
+        <v>282</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F188"/>
+  <autoFilter ref="A1:F189"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Categorize Mary Gerbino Zelle (marketplace bench) and $8.99 CapCut refund
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PkDrCxYQg69AVAk2ernwu3
</commit_message>
<xml_diff>
--- a/reports/September_2026_Expenses.xlsx
+++ b/reports/September_2026_Expenses.xlsx
@@ -1748,7 +1748,7 @@
       </c>
       <c r="C22" s="5" t="n">
         <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A22,'Line Items'!$E$2:$E$195,$B22,'Line Items'!$C$2:$C$195,"Checking")</f>
-        <v>2900.9</v>
+        <v>2890.9</v>
       </c>
       <c r="D22" s="5" t="n">
         <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A22,'Line Items'!$E$2:$E$195,$B22,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="E22" s="5" t="n">
         <f aca="false">C22+D22</f>
-        <v>2930.9</v>
+        <v>2920.9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="C27" s="5" t="n">
         <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A27,'Line Items'!$E$2:$E$195,$B27,'Line Items'!$C$2:$C$195,"Checking")</f>
-        <v>331.53</v>
+        <v>341.53</v>
       </c>
       <c r="D27" s="5" t="n">
         <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A27,'Line Items'!$E$2:$E$195,$B27,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="E27" s="5" t="n">
         <f aca="false">C27+D27</f>
-        <v>384.91</v>
+        <v>394.91</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6299,7 +6299,7 @@
         <v>24</v>
       </c>
       <c r="E191" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F191" s="5" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Expense report: skip card payments filed under a card's sub-category; clean source names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PkDrCxYQg69AVAk2ernwu3
</commit_message>
<xml_diff>
--- a/reports/September_2026_Expenses.xlsx
+++ b/reports/September_2026_Expenses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Line Items" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Line Items'!$A$1:$F$195</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Line Items'!$A$1:$F$194</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="283">
   <si>
     <t xml:space="preserve">Perez Household - 2026-09 Expenses</t>
   </si>
@@ -185,9 +185,6 @@
     <t xml:space="preserve">CC - Ollo</t>
   </si>
   <si>
-    <t xml:space="preserve">CC - Credit 1 (...4838)</t>
-  </si>
-  <si>
     <t xml:space="preserve">CC - Citibank</t>
   </si>
   <si>
@@ -359,7 +356,7 @@
     <t xml:space="preserve">ANNUAL FEE     10/26 THROUGH 10/26</t>
   </si>
   <si>
-    <t xml:space="preserve">Credit One Bank (...4838) (...4838)</t>
+    <t xml:space="preserve">Credit One Bank (...4838)</t>
   </si>
   <si>
     <t xml:space="preserve">LATE FEE</t>
@@ -491,7 +488,7 @@
     <t xml:space="preserve">WM SUPERCENTER #3350 LAS VEGAS NV            09/10</t>
   </si>
   <si>
-    <t xml:space="preserve">Credit One Bank (...4352) (...4352)</t>
+    <t xml:space="preserve">Credit One Bank (...4352)</t>
   </si>
   <si>
     <t xml:space="preserve">GIFTHEALTH*LILLYDIRECT COLUMBUS OH</t>
@@ -777,9 +774,6 @@
   </si>
   <si>
     <t xml:space="preserve">Affirm - Pickleball - installment 2/4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC - Credit 1 (...4838) - checked off as paid</t>
   </si>
   <si>
     <t xml:space="preserve">Cal pizza kitchen</t>
@@ -1381,7 +1375,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -1424,11 +1418,11 @@
         <v>8</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A5,'Line Items'!$E$2:$E$195,$B5,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A5,'Line Items'!$E$2:$E$194,$B5,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>278.91</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A5,'Line Items'!$E$2:$E$195,$B5,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A5,'Line Items'!$E$2:$E$194,$B5,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>310.89</v>
       </c>
       <c r="E5" s="5" t="n">
@@ -1444,11 +1438,11 @@
         <v>9</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A6,'Line Items'!$E$2:$E$195,$B6,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A6,'Line Items'!$E$2:$E$194,$B6,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>401.75</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A6,'Line Items'!$E$2:$E$195,$B6,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A6,'Line Items'!$E$2:$E$194,$B6,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E6" s="5" t="n">
@@ -1464,11 +1458,11 @@
         <v>10</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A7,'Line Items'!$E$2:$E$195,$B7,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A7,'Line Items'!$E$2:$E$194,$B7,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>289.55</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A7,'Line Items'!$E$2:$E$195,$B7,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A7,'Line Items'!$E$2:$E$194,$B7,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
@@ -1484,11 +1478,11 @@
         <v>11</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A8,'Line Items'!$E$2:$E$195,$B8,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A8,'Line Items'!$E$2:$E$194,$B8,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>205.62</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A8,'Line Items'!$E$2:$E$195,$B8,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A8,'Line Items'!$E$2:$E$194,$B8,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
@@ -1504,11 +1498,11 @@
         <v>12</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A9,'Line Items'!$E$2:$E$195,$B9,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A9,'Line Items'!$E$2:$E$194,$B9,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>200</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A9,'Line Items'!$E$2:$E$195,$B9,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A9,'Line Items'!$E$2:$E$194,$B9,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
@@ -1524,11 +1518,11 @@
         <v>13</v>
       </c>
       <c r="C10" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A10,'Line Items'!$E$2:$E$195,$B10,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A10,'Line Items'!$E$2:$E$194,$B10,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>130</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A10,'Line Items'!$E$2:$E$195,$B10,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A10,'Line Items'!$E$2:$E$194,$B10,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E10" s="5" t="n">
@@ -1544,11 +1538,11 @@
         <v>14</v>
       </c>
       <c r="C11" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A11,'Line Items'!$E$2:$E$195,$B11,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A11,'Line Items'!$E$2:$E$194,$B11,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>93.31</v>
       </c>
       <c r="D11" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A11,'Line Items'!$E$2:$E$195,$B11,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A11,'Line Items'!$E$2:$E$194,$B11,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E11" s="5" t="n">
@@ -1564,11 +1558,11 @@
         <v>15</v>
       </c>
       <c r="C12" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A12,'Line Items'!$E$2:$E$195,$B12,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A12,'Line Items'!$E$2:$E$194,$B12,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>59.67</v>
       </c>
       <c r="D12" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A12,'Line Items'!$E$2:$E$195,$B12,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A12,'Line Items'!$E$2:$E$194,$B12,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E12" s="5" t="n">
@@ -1584,11 +1578,11 @@
         <v>16</v>
       </c>
       <c r="C13" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A13,'Line Items'!$E$2:$E$195,$B13,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A13,'Line Items'!$E$2:$E$194,$B13,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>49.72</v>
       </c>
       <c r="D13" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A13,'Line Items'!$E$2:$E$195,$B13,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A13,'Line Items'!$E$2:$E$194,$B13,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
@@ -1604,11 +1598,11 @@
         <v>17</v>
       </c>
       <c r="C14" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A14,'Line Items'!$E$2:$E$195,$B14,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A14,'Line Items'!$E$2:$E$194,$B14,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>48.96</v>
       </c>
       <c r="D14" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A14,'Line Items'!$E$2:$E$195,$B14,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A14,'Line Items'!$E$2:$E$194,$B14,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E14" s="5" t="n">
@@ -1624,11 +1618,11 @@
         <v>18</v>
       </c>
       <c r="C15" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A15,'Line Items'!$E$2:$E$195,$B15,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A15,'Line Items'!$E$2:$E$194,$B15,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>29.98</v>
       </c>
       <c r="D15" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A15,'Line Items'!$E$2:$E$195,$B15,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A15,'Line Items'!$E$2:$E$194,$B15,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E15" s="5" t="n">
@@ -1644,11 +1638,11 @@
         <v>19</v>
       </c>
       <c r="C16" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A16,'Line Items'!$E$2:$E$195,$B16,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A16,'Line Items'!$E$2:$E$194,$B16,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>14.99</v>
       </c>
       <c r="D16" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A16,'Line Items'!$E$2:$E$195,$B16,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A16,'Line Items'!$E$2:$E$194,$B16,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E16" s="5" t="n">
@@ -1664,11 +1658,11 @@
         <v>20</v>
       </c>
       <c r="C17" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A17,'Line Items'!$E$2:$E$195,$B17,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A17,'Line Items'!$E$2:$E$194,$B17,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>14.39</v>
       </c>
       <c r="D17" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A17,'Line Items'!$E$2:$E$195,$B17,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A17,'Line Items'!$E$2:$E$194,$B17,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
@@ -1684,11 +1678,11 @@
         <v>21</v>
       </c>
       <c r="C18" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A18,'Line Items'!$E$2:$E$195,$B18,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A18,'Line Items'!$E$2:$E$194,$B18,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>13.99</v>
       </c>
       <c r="D18" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A18,'Line Items'!$E$2:$E$195,$B18,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A18,'Line Items'!$E$2:$E$194,$B18,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E18" s="5" t="n">
@@ -1704,11 +1698,11 @@
         <v>22</v>
       </c>
       <c r="C19" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A19,'Line Items'!$E$2:$E$195,$B19,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A19,'Line Items'!$E$2:$E$194,$B19,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>13.49</v>
       </c>
       <c r="D19" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A19,'Line Items'!$E$2:$E$195,$B19,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A19,'Line Items'!$E$2:$E$194,$B19,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E19" s="5" t="n">
@@ -1747,11 +1741,11 @@
         <v>25</v>
       </c>
       <c r="C22" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A22,'Line Items'!$E$2:$E$195,$B22,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A22,'Line Items'!$E$2:$E$194,$B22,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>2890.9</v>
       </c>
       <c r="D22" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A22,'Line Items'!$E$2:$E$195,$B22,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A22,'Line Items'!$E$2:$E$194,$B22,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>30</v>
       </c>
       <c r="E22" s="5" t="n">
@@ -1767,11 +1761,11 @@
         <v>26</v>
       </c>
       <c r="C23" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A23,'Line Items'!$E$2:$E$195,$B23,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A23,'Line Items'!$E$2:$E$194,$B23,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>1280.67</v>
       </c>
       <c r="D23" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A23,'Line Items'!$E$2:$E$195,$B23,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A23,'Line Items'!$E$2:$E$194,$B23,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E23" s="5" t="n">
@@ -1787,11 +1781,11 @@
         <v>27</v>
       </c>
       <c r="C24" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A24,'Line Items'!$E$2:$E$195,$B24,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A24,'Line Items'!$E$2:$E$194,$B24,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>762.18</v>
       </c>
       <c r="D24" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A24,'Line Items'!$E$2:$E$195,$B24,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A24,'Line Items'!$E$2:$E$194,$B24,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E24" s="5" t="n">
@@ -1807,11 +1801,11 @@
         <v>28</v>
       </c>
       <c r="C25" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A25,'Line Items'!$E$2:$E$195,$B25,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A25,'Line Items'!$E$2:$E$194,$B25,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>741.55</v>
       </c>
       <c r="D25" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A25,'Line Items'!$E$2:$E$195,$B25,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A25,'Line Items'!$E$2:$E$194,$B25,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E25" s="5" t="n">
@@ -1827,11 +1821,11 @@
         <v>29</v>
       </c>
       <c r="C26" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A26,'Line Items'!$E$2:$E$195,$B26,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A26,'Line Items'!$E$2:$E$194,$B26,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>469.52</v>
       </c>
       <c r="D26" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A26,'Line Items'!$E$2:$E$195,$B26,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A26,'Line Items'!$E$2:$E$194,$B26,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E26" s="5" t="n">
@@ -1847,11 +1841,11 @@
         <v>30</v>
       </c>
       <c r="C27" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A27,'Line Items'!$E$2:$E$195,$B27,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A27,'Line Items'!$E$2:$E$194,$B27,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>341.53</v>
       </c>
       <c r="D27" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A27,'Line Items'!$E$2:$E$195,$B27,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A27,'Line Items'!$E$2:$E$194,$B27,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>53.38</v>
       </c>
       <c r="E27" s="5" t="n">
@@ -1867,11 +1861,11 @@
         <v>31</v>
       </c>
       <c r="C28" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A28,'Line Items'!$E$2:$E$195,$B28,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A28,'Line Items'!$E$2:$E$194,$B28,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D28" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A28,'Line Items'!$E$2:$E$195,$B28,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A28,'Line Items'!$E$2:$E$194,$B28,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>331</v>
       </c>
       <c r="E28" s="5" t="n">
@@ -1887,11 +1881,11 @@
         <v>32</v>
       </c>
       <c r="C29" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A29,'Line Items'!$E$2:$E$195,$B29,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A29,'Line Items'!$E$2:$E$194,$B29,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>21.66</v>
       </c>
       <c r="D29" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A29,'Line Items'!$E$2:$E$195,$B29,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A29,'Line Items'!$E$2:$E$194,$B29,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>304.42</v>
       </c>
       <c r="E29" s="5" t="n">
@@ -1907,11 +1901,11 @@
         <v>33</v>
       </c>
       <c r="C30" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A30,'Line Items'!$E$2:$E$195,$B30,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A30,'Line Items'!$E$2:$E$194,$B30,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>211.4</v>
       </c>
       <c r="D30" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A30,'Line Items'!$E$2:$E$195,$B30,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A30,'Line Items'!$E$2:$E$194,$B30,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>67.49</v>
       </c>
       <c r="E30" s="5" t="n">
@@ -1927,11 +1921,11 @@
         <v>34</v>
       </c>
       <c r="C31" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A31,'Line Items'!$E$2:$E$195,$B31,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A31,'Line Items'!$E$2:$E$194,$B31,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>242.45</v>
       </c>
       <c r="D31" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A31,'Line Items'!$E$2:$E$195,$B31,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A31,'Line Items'!$E$2:$E$194,$B31,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E31" s="5" t="n">
@@ -1947,11 +1941,11 @@
         <v>35</v>
       </c>
       <c r="C32" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A32,'Line Items'!$E$2:$E$195,$B32,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A32,'Line Items'!$E$2:$E$194,$B32,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>232.71</v>
       </c>
       <c r="D32" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A32,'Line Items'!$E$2:$E$195,$B32,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A32,'Line Items'!$E$2:$E$194,$B32,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E32" s="5" t="n">
@@ -1967,11 +1961,11 @@
         <v>36</v>
       </c>
       <c r="C33" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A33,'Line Items'!$E$2:$E$195,$B33,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A33,'Line Items'!$E$2:$E$194,$B33,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>175.94</v>
       </c>
       <c r="D33" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A33,'Line Items'!$E$2:$E$195,$B33,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A33,'Line Items'!$E$2:$E$194,$B33,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E33" s="5" t="n">
@@ -1987,11 +1981,11 @@
         <v>37</v>
       </c>
       <c r="C34" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A34,'Line Items'!$E$2:$E$195,$B34,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A34,'Line Items'!$E$2:$E$194,$B34,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>93.04</v>
       </c>
       <c r="D34" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A34,'Line Items'!$E$2:$E$195,$B34,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A34,'Line Items'!$E$2:$E$194,$B34,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E34" s="5" t="n">
@@ -2007,11 +2001,11 @@
         <v>38</v>
       </c>
       <c r="C35" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A35,'Line Items'!$E$2:$E$195,$B35,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A35,'Line Items'!$E$2:$E$194,$B35,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>47.93</v>
       </c>
       <c r="D35" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A35,'Line Items'!$E$2:$E$195,$B35,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A35,'Line Items'!$E$2:$E$194,$B35,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E35" s="5" t="n">
@@ -2027,11 +2021,11 @@
         <v>39</v>
       </c>
       <c r="C36" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A36,'Line Items'!$E$2:$E$195,$B36,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A36,'Line Items'!$E$2:$E$194,$B36,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D36" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A36,'Line Items'!$E$2:$E$195,$B36,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A36,'Line Items'!$E$2:$E$194,$B36,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>40</v>
       </c>
       <c r="E36" s="5" t="n">
@@ -2047,11 +2041,11 @@
         <v>40</v>
       </c>
       <c r="C37" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A37,'Line Items'!$E$2:$E$195,$B37,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A37,'Line Items'!$E$2:$E$194,$B37,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>40</v>
       </c>
       <c r="D37" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A37,'Line Items'!$E$2:$E$195,$B37,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A37,'Line Items'!$E$2:$E$194,$B37,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E37" s="5" t="n">
@@ -2067,11 +2061,11 @@
         <v>41</v>
       </c>
       <c r="C38" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A38,'Line Items'!$E$2:$E$195,$B38,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A38,'Line Items'!$E$2:$E$194,$B38,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>7.8</v>
       </c>
       <c r="D38" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A38,'Line Items'!$E$2:$E$195,$B38,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A38,'Line Items'!$E$2:$E$194,$B38,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E38" s="5" t="n">
@@ -2087,11 +2081,11 @@
         <v>42</v>
       </c>
       <c r="C39" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A39,'Line Items'!$E$2:$E$195,$B39,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A39,'Line Items'!$E$2:$E$194,$B39,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>7</v>
       </c>
       <c r="D39" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A39,'Line Items'!$E$2:$E$195,$B39,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A39,'Line Items'!$E$2:$E$194,$B39,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E39" s="5" t="n">
@@ -2130,11 +2124,11 @@
         <v>45</v>
       </c>
       <c r="C42" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A42,'Line Items'!$E$2:$E$195,$B42,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A42,'Line Items'!$E$2:$E$194,$B42,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>1120.71</v>
       </c>
       <c r="D42" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A42,'Line Items'!$E$2:$E$195,$B42,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A42,'Line Items'!$E$2:$E$194,$B42,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E42" s="5" t="n">
@@ -2150,11 +2144,11 @@
         <v>46</v>
       </c>
       <c r="C43" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A43,'Line Items'!$E$2:$E$195,$B43,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A43,'Line Items'!$E$2:$E$194,$B43,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>709.9</v>
       </c>
       <c r="D43" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A43,'Line Items'!$E$2:$E$195,$B43,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A43,'Line Items'!$E$2:$E$194,$B43,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E43" s="5" t="n">
@@ -2170,11 +2164,11 @@
         <v>47</v>
       </c>
       <c r="C44" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A44,'Line Items'!$E$2:$E$195,$B44,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A44,'Line Items'!$E$2:$E$194,$B44,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>706.36</v>
       </c>
       <c r="D44" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A44,'Line Items'!$E$2:$E$195,$B44,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A44,'Line Items'!$E$2:$E$194,$B44,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E44" s="5" t="n">
@@ -2190,11 +2184,11 @@
         <v>48</v>
       </c>
       <c r="C45" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A45,'Line Items'!$E$2:$E$195,$B45,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A45,'Line Items'!$E$2:$E$194,$B45,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>500</v>
       </c>
       <c r="D45" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A45,'Line Items'!$E$2:$E$195,$B45,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A45,'Line Items'!$E$2:$E$194,$B45,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E45" s="5" t="n">
@@ -2210,11 +2204,11 @@
         <v>49</v>
       </c>
       <c r="C46" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A46,'Line Items'!$E$2:$E$195,$B46,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A46,'Line Items'!$E$2:$E$194,$B46,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>214.19</v>
       </c>
       <c r="D46" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A46,'Line Items'!$E$2:$E$195,$B46,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A46,'Line Items'!$E$2:$E$194,$B46,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E46" s="5" t="n">
@@ -2230,11 +2224,11 @@
         <v>50</v>
       </c>
       <c r="C47" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A47,'Line Items'!$E$2:$E$195,$B47,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A47,'Line Items'!$E$2:$E$194,$B47,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>150.4</v>
       </c>
       <c r="D47" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A47,'Line Items'!$E$2:$E$195,$B47,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A47,'Line Items'!$E$2:$E$194,$B47,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>0</v>
       </c>
       <c r="E47" s="5" t="n">
@@ -2250,11 +2244,11 @@
         <v>51</v>
       </c>
       <c r="C48" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A48,'Line Items'!$E$2:$E$195,$B48,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A48,'Line Items'!$E$2:$E$194,$B48,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D48" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A48,'Line Items'!$E$2:$E$195,$B48,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A48,'Line Items'!$E$2:$E$194,$B48,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>46.5</v>
       </c>
       <c r="E48" s="5" t="n">
@@ -2270,11 +2264,11 @@
         <v>52</v>
       </c>
       <c r="C49" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A49,'Line Items'!$E$2:$E$195,$B49,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A49,'Line Items'!$E$2:$E$194,$B49,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D49" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A49,'Line Items'!$E$2:$E$195,$B49,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A49,'Line Items'!$E$2:$E$194,$B49,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
         <v>27</v>
       </c>
       <c r="E49" s="5" t="n">
@@ -2290,16 +2284,16 @@
         <v>53</v>
       </c>
       <c r="C50" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A50,'Line Items'!$E$2:$E$195,$B50,'Line Items'!$C$2:$C$195,"Checking")</f>
-        <v>24.94</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A50,'Line Items'!$E$2:$E$194,$B50,'Line Items'!$C$2:$C$194,"Checking")</f>
+        <v>0</v>
       </c>
       <c r="D50" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A50,'Line Items'!$E$2:$E$195,$B50,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
-        <v>0</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A50,'Line Items'!$E$2:$E$194,$B50,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
+        <v>15.9</v>
       </c>
       <c r="E50" s="5" t="n">
         <f aca="false">C50+D50</f>
-        <v>24.94</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2310,126 +2304,111 @@
         <v>54</v>
       </c>
       <c r="C51" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A51,'Line Items'!$E$2:$E$195,$B51,'Line Items'!$C$2:$C$195,"Checking")</f>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A51,'Line Items'!$E$2:$E$194,$B51,'Line Items'!$C$2:$C$194,"Checking")</f>
         <v>0</v>
       </c>
       <c r="D51" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A51,'Line Items'!$E$2:$E$195,$B51,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
-        <v>15.9</v>
+        <f aca="false">SUMIFS('Line Items'!$F$2:$F$194,'Line Items'!$D$2:$D$194,$A51,'Line Items'!$E$2:$E$194,$B51,'Line Items'!$C$2:$C$194,"&lt;&gt;Checking")</f>
+        <v>5.68</v>
       </c>
       <c r="E51" s="5" t="n">
         <f aca="false">C51+D51</f>
-        <v>15.9</v>
+        <v>5.68</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B52" s="4" t="s">
+      <c r="A52" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C52" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A52,'Line Items'!$E$2:$E$195,$B52,'Line Items'!$C$2:$C$195,"Checking")</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="5" t="n">
-        <f aca="false">SUMIFS('Line Items'!$F$2:$F$195,'Line Items'!$D$2:$D$195,$A52,'Line Items'!$E$2:$E$195,$B52,'Line Items'!$C$2:$C$195,"&lt;&gt;Checking")</f>
-        <v>5.68</v>
-      </c>
-      <c r="E52" s="5" t="n">
-        <f aca="false">C52+D52</f>
-        <v>5.68</v>
+      <c r="B52" s="6"/>
+      <c r="C52" s="7" t="n">
+        <f aca="false">SUM(C42:C51)</f>
+        <v>3401.56</v>
+      </c>
+      <c r="D52" s="7" t="n">
+        <f aca="false">SUM(D42:D51)</f>
+        <v>95.08</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <f aca="false">SUM(E42:E51)</f>
+        <v>3496.64</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="s">
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B53" s="6"/>
-      <c r="C53" s="7" t="n">
-        <f aca="false">SUM(C42:C52)</f>
-        <v>3426.5</v>
-      </c>
-      <c r="D53" s="7" t="n">
-        <f aca="false">SUM(D42:D52)</f>
-        <v>95.08</v>
-      </c>
-      <c r="E53" s="7" t="n">
-        <f aca="false">SUM(E42:E52)</f>
-        <v>3521.58</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C54" s="8"/>
-      <c r="D54" s="8"/>
-      <c r="E54" s="8"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="10" t="n">
+        <f aca="false">C20+C40+C52</f>
+        <v>12812.17</v>
+      </c>
+      <c r="D54" s="10" t="n">
+        <f aca="false">D20+D40+D52</f>
+        <v>1232.26</v>
+      </c>
+      <c r="E54" s="10" t="n">
+        <f aca="false">E20+E40+E52</f>
+        <v>14044.43</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="9" t="s">
+      <c r="B55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="9"/>
-      <c r="C55" s="10" t="n">
-        <f aca="false">C20+C40+C53</f>
-        <v>12837.11</v>
-      </c>
-      <c r="D55" s="10" t="n">
-        <f aca="false">D20+D40+D53</f>
-        <v>1232.26</v>
-      </c>
-      <c r="E55" s="10" t="n">
-        <f aca="false">E20+E40+E53</f>
-        <v>14069.37</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="2" t="s">
+      <c r="E55" s="2" t="str">
+        <f aca="false">IF(ROUND(E54-'Line Items'!F195,2)=0,"OK","MISMATCH")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="E56" s="2" t="str">
-        <f aca="false">IF(ROUND(E55-'Line Items'!F196,2)=0,"OK","MISMATCH")</f>
-        <v>OK</v>
-      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="4" t="s">
         <v>59</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>10.74</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>10.74</v>
+        <v>13.06</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E60" s="5" t="n">
-        <v>13.06</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="11" t="s">
+      <c r="E60" s="12" t="n">
+        <f aca="false">SUM(E58:E59)</f>
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E61" s="12" t="n">
-        <f aca="false">SUM(E59:E60)</f>
-        <v>23.8</v>
-      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="13" t="s">
+      <c r="A63" s="14" t="s">
         <v>65</v>
       </c>
     </row>
@@ -2451,11 +2430,6 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="14" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2474,7 +2448,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F198"/>
+  <dimension ref="A1:F197"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -2487,13 +2461,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -2502,18 +2476,18 @@
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>76</v>
-      </c>
       <c r="C2" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>24</v>
@@ -2527,13 +2501,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>24</v>
@@ -2547,13 +2521,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>24</v>
@@ -2567,13 +2541,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>24</v>
@@ -2587,13 +2561,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>82</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>24</v>
@@ -2607,13 +2581,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>82</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>24</v>
@@ -2627,13 +2601,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>84</v>
-      </c>
       <c r="C8" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>24</v>
@@ -2647,13 +2621,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>24</v>
@@ -2667,13 +2641,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>24</v>
@@ -2687,13 +2661,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>24</v>
@@ -2707,13 +2681,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>24</v>
@@ -2727,13 +2701,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>24</v>
@@ -2747,13 +2721,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>24</v>
@@ -2767,13 +2741,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>24</v>
@@ -2787,13 +2761,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>92</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>93</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>24</v>
@@ -2807,13 +2781,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>95</v>
-      </c>
       <c r="C17" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>24</v>
@@ -2827,13 +2801,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>24</v>
@@ -2847,13 +2821,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>24</v>
@@ -2867,13 +2841,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>24</v>
@@ -2887,13 +2861,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>24</v>
@@ -2907,13 +2881,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>24</v>
@@ -2927,13 +2901,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>24</v>
@@ -2947,13 +2921,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>24</v>
@@ -2967,13 +2941,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>104</v>
-      </c>
       <c r="C25" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>24</v>
@@ -2987,13 +2961,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>44</v>
@@ -3007,13 +2981,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>24</v>
@@ -3027,13 +3001,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>24</v>
@@ -3047,13 +3021,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>24</v>
@@ -3067,13 +3041,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>24</v>
@@ -3087,13 +3061,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>110</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>111</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>44</v>
@@ -3107,13 +3081,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>44</v>
@@ -3127,13 +3101,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>114</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>44</v>
@@ -3147,13 +3121,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>116</v>
-      </c>
       <c r="C34" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>24</v>
@@ -3167,13 +3141,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>118</v>
-      </c>
       <c r="C35" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>24</v>
@@ -3187,13 +3161,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>24</v>
@@ -3207,13 +3181,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>24</v>
@@ -3227,13 +3201,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>24</v>
@@ -3247,13 +3221,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>7</v>
@@ -3267,13 +3241,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>44</v>
@@ -3287,13 +3261,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>24</v>
@@ -3307,13 +3281,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>24</v>
@@ -3327,13 +3301,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>24</v>
@@ -3347,13 +3321,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>24</v>
@@ -3367,13 +3341,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>24</v>
@@ -3387,13 +3361,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>24</v>
@@ -3407,13 +3381,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>24</v>
@@ -3427,13 +3401,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>24</v>
@@ -3447,13 +3421,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>7</v>
@@ -3467,13 +3441,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>24</v>
@@ -3487,13 +3461,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>24</v>
@@ -3507,13 +3481,13 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>44</v>
@@ -3527,13 +3501,13 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>24</v>
@@ -3547,13 +3521,13 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>24</v>
@@ -3567,13 +3541,13 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>24</v>
@@ -3587,13 +3561,13 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>7</v>
@@ -3607,13 +3581,13 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>24</v>
@@ -3627,13 +3601,13 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>24</v>
@@ -3647,13 +3621,13 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>24</v>
@@ -3667,13 +3641,13 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>24</v>
@@ -3687,13 +3661,13 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B61" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>144</v>
-      </c>
       <c r="C61" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>24</v>
@@ -3707,13 +3681,13 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>24</v>
@@ -3727,13 +3701,13 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>24</v>
@@ -3747,13 +3721,13 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>7</v>
@@ -3767,13 +3741,13 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>24</v>
@@ -3787,13 +3761,13 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>24</v>
@@ -3807,13 +3781,13 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B67" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C67" s="4" t="s">
         <v>150</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>151</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>24</v>
@@ -3827,13 +3801,13 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B68" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>153</v>
-      </c>
       <c r="C68" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>24</v>
@@ -3847,13 +3821,13 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>24</v>
@@ -3867,13 +3841,13 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>44</v>
@@ -3887,13 +3861,13 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B71" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C71" s="4" t="s">
         <v>156</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>157</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>24</v>
@@ -3907,13 +3881,13 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B72" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B72" s="4" t="s">
-        <v>159</v>
-      </c>
       <c r="C72" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>44</v>
@@ -3927,13 +3901,13 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>24</v>
@@ -3947,13 +3921,13 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>44</v>
@@ -3967,13 +3941,13 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>24</v>
@@ -3987,13 +3961,13 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>24</v>
@@ -4007,13 +3981,13 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>24</v>
@@ -4027,13 +4001,13 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>7</v>
@@ -4047,13 +4021,13 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>24</v>
@@ -4067,13 +4041,13 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B80" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B80" s="4" t="s">
-        <v>168</v>
-      </c>
       <c r="C80" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>24</v>
@@ -4087,13 +4061,13 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B81" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B81" s="4" t="s">
-        <v>170</v>
-      </c>
       <c r="C81" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>44</v>
@@ -4107,13 +4081,13 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>24</v>
@@ -4127,13 +4101,13 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>44</v>
@@ -4147,13 +4121,13 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>24</v>
@@ -4167,13 +4141,13 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>24</v>
@@ -4187,13 +4161,13 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>24</v>
@@ -4207,13 +4181,13 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B87" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B87" s="4" t="s">
+      <c r="C87" s="4" t="s">
         <v>176</v>
-      </c>
-      <c r="C87" s="4" t="s">
-        <v>177</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>24</v>
@@ -4227,13 +4201,13 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D88" s="4" t="s">
         <v>24</v>
@@ -4247,13 +4221,13 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>24</v>
@@ -4267,13 +4241,13 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>24</v>
@@ -4287,13 +4261,13 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B91" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="B91" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="C91" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>44</v>
@@ -4307,13 +4281,13 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>24</v>
@@ -4327,13 +4301,13 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>7</v>
@@ -4347,13 +4321,13 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>24</v>
@@ -4367,13 +4341,13 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D95" s="4" t="s">
         <v>24</v>
@@ -4387,13 +4361,13 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>24</v>
@@ -4407,13 +4381,13 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>24</v>
@@ -4427,13 +4401,13 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>24</v>
@@ -4447,13 +4421,13 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>24</v>
@@ -4467,13 +4441,13 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>7</v>
@@ -4487,13 +4461,13 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>7</v>
@@ -4507,13 +4481,13 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B102" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B102" s="4" t="s">
-        <v>193</v>
-      </c>
       <c r="C102" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D102" s="4" t="s">
         <v>24</v>
@@ -4527,13 +4501,13 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D103" s="4" t="s">
         <v>24</v>
@@ -4547,13 +4521,13 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D104" s="4" t="s">
         <v>24</v>
@@ -4567,13 +4541,13 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B105" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B105" s="4" t="s">
-        <v>196</v>
-      </c>
       <c r="C105" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D105" s="4" t="s">
         <v>24</v>
@@ -4587,13 +4561,13 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B106" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B106" s="4" t="s">
-        <v>196</v>
-      </c>
       <c r="C106" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>24</v>
@@ -4607,13 +4581,13 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B107" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B107" s="4" t="s">
-        <v>196</v>
-      </c>
       <c r="C107" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>24</v>
@@ -4627,13 +4601,13 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D108" s="4" t="s">
         <v>24</v>
@@ -4647,13 +4621,13 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D109" s="4" t="s">
         <v>7</v>
@@ -4667,19 +4641,19 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D110" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F110" s="5" t="n">
         <v>5.68</v>
@@ -4687,13 +4661,13 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B111" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="B111" s="4" t="s">
-        <v>201</v>
-      </c>
       <c r="C111" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D111" s="4" t="s">
         <v>44</v>
@@ -4707,13 +4681,13 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D112" s="4" t="s">
         <v>44</v>
@@ -4727,13 +4701,13 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D113" s="4" t="s">
         <v>24</v>
@@ -4747,13 +4721,13 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D114" s="4" t="s">
         <v>24</v>
@@ -4767,13 +4741,13 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D115" s="4" t="s">
         <v>24</v>
@@ -4787,13 +4761,13 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D116" s="4" t="s">
         <v>24</v>
@@ -4807,13 +4781,13 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B117" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>24</v>
@@ -4827,13 +4801,13 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D118" s="4" t="s">
         <v>24</v>
@@ -4847,13 +4821,13 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>24</v>
@@ -4867,19 +4841,19 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F120" s="5" t="n">
         <v>15.9</v>
@@ -4887,13 +4861,13 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B121" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="B121" s="4" t="s">
-        <v>211</v>
-      </c>
       <c r="C121" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D121" s="4" t="s">
         <v>44</v>
@@ -4907,13 +4881,13 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D122" s="4" t="s">
         <v>24</v>
@@ -4927,13 +4901,13 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>24</v>
@@ -4947,13 +4921,13 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D124" s="4" t="s">
         <v>24</v>
@@ -4967,13 +4941,13 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>24</v>
@@ -4987,13 +4961,13 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B126" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="B126" s="4" t="s">
-        <v>216</v>
-      </c>
       <c r="C126" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>44</v>
@@ -5007,13 +4981,13 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D127" s="4" t="s">
         <v>7</v>
@@ -5027,13 +5001,13 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D128" s="4" t="s">
         <v>7</v>
@@ -5047,13 +5021,13 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D129" s="4" t="s">
         <v>24</v>
@@ -5067,13 +5041,13 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D130" s="4" t="s">
         <v>24</v>
@@ -5087,13 +5061,13 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D131" s="4" t="s">
         <v>24</v>
@@ -5107,13 +5081,13 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D132" s="4" t="s">
         <v>24</v>
@@ -5127,13 +5101,13 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D133" s="4" t="s">
         <v>24</v>
@@ -5147,13 +5121,13 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D134" s="4" t="s">
         <v>24</v>
@@ -5167,13 +5141,13 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B135" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="B135" s="4" t="s">
-        <v>226</v>
-      </c>
       <c r="C135" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D135" s="4" t="s">
         <v>7</v>
@@ -5187,13 +5161,13 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D136" s="4" t="s">
         <v>24</v>
@@ -5207,13 +5181,13 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>24</v>
@@ -5227,13 +5201,13 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B138" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="B138" s="4" t="s">
-        <v>230</v>
-      </c>
       <c r="C138" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D138" s="4" t="s">
         <v>24</v>
@@ -5247,13 +5221,13 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D139" s="4" t="s">
         <v>7</v>
@@ -5267,13 +5241,13 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D140" s="4" t="s">
         <v>7</v>
@@ -5287,13 +5261,13 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>24</v>
@@ -5307,13 +5281,13 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D142" s="4" t="s">
         <v>24</v>
@@ -5327,13 +5301,13 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D143" s="4" t="s">
         <v>24</v>
@@ -5347,13 +5321,13 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D144" s="4" t="s">
         <v>24</v>
@@ -5367,13 +5341,13 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D145" s="4" t="s">
         <v>24</v>
@@ -5387,13 +5361,13 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D146" s="4" t="s">
         <v>24</v>
@@ -5407,13 +5381,13 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B147" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="B147" s="4" t="s">
-        <v>238</v>
-      </c>
       <c r="C147" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D147" s="4" t="s">
         <v>44</v>
@@ -5427,13 +5401,13 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D148" s="4" t="s">
         <v>24</v>
@@ -5447,13 +5421,13 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D149" s="4" t="s">
         <v>24</v>
@@ -5467,13 +5441,13 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B150" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="B150" s="4" t="s">
-        <v>241</v>
-      </c>
       <c r="C150" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D150" s="4" t="s">
         <v>44</v>
@@ -5487,13 +5461,13 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D151" s="4" t="s">
         <v>7</v>
@@ -5507,13 +5481,13 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D152" s="4" t="s">
         <v>7</v>
@@ -5527,13 +5501,13 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D153" s="4" t="s">
         <v>24</v>
@@ -5547,13 +5521,13 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D154" s="4" t="s">
         <v>24</v>
@@ -5567,13 +5541,13 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D155" s="4" t="s">
         <v>24</v>
@@ -5587,13 +5561,13 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D156" s="4" t="s">
         <v>44</v>
@@ -5607,13 +5581,13 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D157" s="4" t="s">
         <v>44</v>
@@ -5627,13 +5601,13 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B158" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D158" s="4" t="s">
         <v>7</v>
@@ -5647,13 +5621,13 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D159" s="4" t="s">
         <v>7</v>
@@ -5667,13 +5641,13 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D160" s="4" t="s">
         <v>24</v>
@@ -5687,13 +5661,13 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D161" s="4" t="s">
         <v>24</v>
@@ -5707,13 +5681,13 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D162" s="4" t="s">
         <v>44</v>
@@ -5727,53 +5701,53 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D163" s="4" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="E163" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F163" s="5" t="n">
-        <v>24.94</v>
+        <v>109.77</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D164" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E164" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F164" s="5" t="n">
-        <v>109.77</v>
+        <v>8.99</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D165" s="4" t="s">
         <v>24</v>
@@ -5782,38 +5756,38 @@
         <v>25</v>
       </c>
       <c r="F165" s="5" t="n">
-        <v>8.99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D166" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E166" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F166" s="5" t="n">
-        <v>96</v>
+        <v>139.14</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D167" s="4" t="s">
         <v>24</v>
@@ -5822,118 +5796,118 @@
         <v>26</v>
       </c>
       <c r="F167" s="5" t="n">
-        <v>139.14</v>
+        <v>66.45</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D168" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E168" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F168" s="5" t="n">
-        <v>66.45</v>
+        <v>19.99</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C169" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D169" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E169" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F169" s="5" t="n">
-        <v>19.99</v>
+        <v>81.76</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C170" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D170" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E170" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F170" s="5" t="n">
-        <v>81.76</v>
+        <v>130.88</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D171" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E171" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F171" s="5" t="n">
-        <v>130.88</v>
+        <v>94.83</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D172" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E172" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F172" s="5" t="n">
-        <v>94.83</v>
+        <v>165.82</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D173" s="4" t="s">
         <v>24</v>
@@ -5942,138 +5916,138 @@
         <v>28</v>
       </c>
       <c r="F173" s="5" t="n">
-        <v>165.82</v>
+        <v>29.25</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D174" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E174" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F174" s="5" t="n">
-        <v>29.25</v>
+        <v>-180.49</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D175" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E175" s="4" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F175" s="5" t="n">
-        <v>-180.49</v>
+        <v>20</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D176" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E176" s="4" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F176" s="5" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="4" t="s">
-        <v>62</v>
+        <v>264</v>
       </c>
       <c r="B177" s="4" t="s">
         <v>265</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D177" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E177" s="4" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="F177" s="5" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="B178" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="B178" s="4" t="s">
-        <v>267</v>
-      </c>
       <c r="C178" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D178" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E178" s="4" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="F178" s="5" t="n">
-        <v>7</v>
+        <v>11.58</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D179" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E179" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F179" s="5" t="n">
-        <v>11.58</v>
+        <v>40.86</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D180" s="4" t="s">
         <v>24</v>
@@ -6082,18 +6056,18 @@
         <v>26</v>
       </c>
       <c r="F180" s="5" t="n">
-        <v>40.86</v>
+        <v>55.29</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D181" s="4" t="s">
         <v>24</v>
@@ -6102,158 +6076,158 @@
         <v>26</v>
       </c>
       <c r="F181" s="5" t="n">
-        <v>55.29</v>
+        <v>34.84</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C182" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D182" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E182" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="F182" s="5" t="n">
-        <v>34.84</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D183" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E183" s="4" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="F183" s="5" t="n">
-        <v>7.8</v>
+        <v>55</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="4" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="B184" s="4" t="s">
         <v>272</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D184" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E184" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B185" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="B185" s="4" t="s">
-        <v>274</v>
-      </c>
       <c r="C185" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D185" s="4" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="E185" s="4" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>60</v>
+        <v>39.33</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>275</v>
+        <v>115</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D186" s="4" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="E186" s="4" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>39.33</v>
+        <v>78.32</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>116</v>
+        <v>274</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D187" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E187" s="4" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F187" s="5" t="n">
-        <v>78.32</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D188" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E188" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F188" s="5" t="n">
-        <v>31.8</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D189" s="4" t="s">
         <v>24</v>
@@ -6262,145 +6236,125 @@
         <v>25</v>
       </c>
       <c r="F189" s="5" t="n">
-        <v>0.01</v>
+        <v>-19.99</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C190" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D190" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E190" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F190" s="5" t="n">
-        <v>-19.99</v>
+        <v>10</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D191" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E191" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F191" s="5" t="n">
-        <v>10</v>
+        <v>30.33</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C192" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D192" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E192" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F192" s="5" t="n">
-        <v>30.33</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D193" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E193" s="4" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="F193" s="5" t="n">
-        <v>9.99</v>
+        <v>161.81</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B194" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="C194" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D194" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E194" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F194" s="5" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E195" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F195" s="12" t="n">
+        <f aca="false">SUM(F2:F194)</f>
+        <v>14044.43</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="C194" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D194" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E194" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F194" s="5" t="n">
-        <v>161.81</v>
-      </c>
-    </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A195" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="B195" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="C195" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D195" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E195" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F195" s="5" t="n">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E196" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="F196" s="12" t="n">
-        <f aca="false">SUM(F2:F195)</f>
-        <v>14069.37</v>
-      </c>
-    </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A198" s="2" t="s">
-        <v>284</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F195"/>
+  <autoFilter ref="A1:F194"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>